<commit_message>
Refactor code structure for improved readability and maintainability; removed redundant code blocks and optimized existing functions.
</commit_message>
<xml_diff>
--- a/sales_rep_analysis_feb2026.xlsx
+++ b/sales_rep_analysis_feb2026.xlsx
@@ -21,11 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +52,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
     <font>
@@ -58,7 +64,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -79,14 +85,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0027AE60"/>
-        <bgColor rgb="0027AE60"/>
+        <fgColor rgb="008E44AD"/>
+        <bgColor rgb="008E44AD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008E44AD"/>
-        <bgColor rgb="008E44AD"/>
+        <fgColor rgb="00D5F5E3"/>
+        <bgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+        <bgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0016A085"/>
+        <bgColor rgb="0016A085"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF3CF"/>
+        <bgColor rgb="00FCF3CF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0027AE60"/>
+        <bgColor rgb="0027AE60"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,17 +148,42 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,7 +674,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Week 1 vs Week 2 vs Week 3 Sales</a:t>
+              <a:t>Week 1 vs Week 2 vs Week 3 vs Week 4 Sales</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -698,6 +753,30 @@
           <val>
             <numRef>
               <f>'Charts'!$D$37:$D$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!E36</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$37:$A$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$E$37:$E$43</f>
             </numRef>
           </val>
         </ser>
@@ -1647,7 +1726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1655,6 +1734,8 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1667,14 +1748,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BOMAS  - February 1-21, 2026</t>
+          <t>BOMAS  - February 1-28, 2026 (Full Month)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Generated: 2026-02-27 15:54:26</t>
+          <t>Generated: 2026-03-01 18:47:35</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1785,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>49669737</v>
+        <v>65670608</v>
       </c>
     </row>
     <row r="8">
@@ -1714,7 +1795,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>4345944.0136</v>
+        <v>5765161.453199999</v>
       </c>
     </row>
     <row r="9">
@@ -1724,17 +1805,17 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.08749681951406346</v>
+        <v>0.08778906772417884</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Daily Average (18 days)</t>
+          <t>Daily Average (24 days)</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>2759429.833333333</v>
+        <v>2736275.333333333</v>
       </c>
     </row>
     <row r="11">
@@ -1841,39 +1922,530 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>W1→W2 Change</t>
+          <t>Week 4 (Feb 23-28)</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>5798168</v>
+        <v>16000871</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>285145.9452</v>
+        <v>1419217.4396</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>-0.01318810373433341</v>
+        <v>0.08869626157226067</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>966361.3333333334</v>
+        <v>2666811.833333333</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>W1→W2 Change</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>5798168</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>285145.9452</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>-0.01318810373433341</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>966361.3333333334</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>W2→W3 Change</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B21" s="6" t="n">
         <v>-4727875</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C21" s="6" t="n">
         <v>-282664.3688000001</v>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D21" s="7" t="n">
         <v>0.006733216360186409</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E21" s="6" t="n">
         <v>-787979.1666666666</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>W3→W4 Change</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>663486</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>63963.69920000038</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.0003334969679947009</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>110581</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY TARGET PERFORMANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Variance</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Variance %</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>OVERALL SHOP</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>65670608</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>5670608</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <v>0.09451013333333332</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>✓ ACHIEVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>GENERAL HARDWARE</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="n">
+        <v>47000000</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>57622740</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>10622740</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <v>0.226015744680851</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>✓ ACHIEVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>PAINTS</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>5807571</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>-1192429</v>
+      </c>
+      <c r="E29" s="16" t="n">
+        <v>-0.170347</v>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>✗ MISSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>PLUMBING</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="C30" s="15" t="n">
+        <v>1777021</v>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>-2222979</v>
+      </c>
+      <c r="E30" s="16" t="n">
+        <v>-0.55574475</v>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>✗ MISSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>ELECTRICALS</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="C31" s="15" t="n">
+        <v>463276</v>
+      </c>
+      <c r="D31" s="15" t="n">
+        <v>-1536724</v>
+      </c>
+      <c r="E31" s="16" t="n">
+        <v>-0.7683620000000001</v>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>✗ MISSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>CUMULATIVE TARGET TRACKING</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t>Week Sales</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Cumulative</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="inlineStr">
+        <is>
+          <t>% of Target</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>Expected %</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>Pace</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>14267092</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <v>14267092</v>
+      </c>
+      <c r="D36" s="19" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>✗ Behind</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="n">
+        <v>20065260</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <v>34332352</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <v>0.5720000000000001</v>
+      </c>
+      <c r="E37" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>✓ Ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>15337385</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <v>49669737</v>
+      </c>
+      <c r="D38" s="20" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="E38" s="20" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>✓ Ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>16000871</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <v>65670608</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>✓ Ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>CATEGORY CONTRIBUTION %</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Share of total sales per week</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Week 1</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>Week 2</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>Week 3</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>Week 4</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>Full Month</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>Trend (W1→W4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>GENERAL HARDWARE</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>0.8540000000000001</v>
+      </c>
+      <c r="C45" s="7" t="n">
+        <v>0.9079999999999999</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>0.8640000000000001</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>0.8740000000000001</v>
+      </c>
+      <c r="F45" s="7" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>↑ Growing (+2.0pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="23" t="inlineStr">
+        <is>
+          <t>PAINTS</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="C46" s="7" t="n">
+        <v>0.06900000000000001</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>0.095</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>0.08800000000000001</v>
+      </c>
+      <c r="G46" s="24" t="inlineStr">
+        <is>
+          <t>→ Stable (+0.0pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>PLUMBING</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>0.044</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="F47" s="7" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>↓ Shrinking (-2.2pp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>ELECTRICALS</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="F48" s="7" t="n">
+        <v>0.006999999999999999</v>
+      </c>
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>→ Stable (+0.1pp)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1902,47 +2474,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="18" t="inlineStr">
         <is>
           <t>Rep Name</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="18" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="18" t="inlineStr">
         <is>
           <t>Total Sales</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="18" t="inlineStr">
         <is>
           <t>Total Profit</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="18" t="inlineStr">
         <is>
           <t>Margin %</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="18" t="inlineStr">
         <is>
           <t>Items Sold</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="18" t="inlineStr">
         <is>
           <t>Margin Rank</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="18" t="inlineStr">
         <is>
           <t>Week Improvement %</t>
         </is>
@@ -1963,22 +2535,22 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>19339020</v>
+        <v>25230250</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>1149098.9116</v>
+        <v>1493076.368</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>0.0594186733143665</v>
-      </c>
-      <c r="G2" s="10" t="n">
-        <v>22606</v>
+        <v>0.05917802510874843</v>
+      </c>
+      <c r="G2" s="25" t="n">
+        <v>29108</v>
       </c>
       <c r="H2" s="5" t="n">
         <v>7</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>-0.1668807939787459</v>
+        <v>0.04614229004054952</v>
       </c>
     </row>
     <row r="3">
@@ -1996,22 +2568,22 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>9453025</v>
+        <v>13451533</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>763497.9292</v>
+        <v>1123301.2308</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0.08076757748974535</v>
-      </c>
-      <c r="G3" s="10" t="n">
-        <v>12927</v>
+        <v>0.08350730216399871</v>
+      </c>
+      <c r="G3" s="25" t="n">
+        <v>18368.5</v>
       </c>
       <c r="H3" s="5" t="n">
         <v>6</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>0.5974423970194863</v>
+        <v>0.7505299517986841</v>
       </c>
     </row>
     <row r="4">
@@ -2029,22 +2601,22 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>8456260</v>
+        <v>11367285</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>842095.0399999998</v>
+        <v>1063081.7332</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>0.09958244424840293</v>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>10636</v>
+        <v>0.09352116474602334</v>
+      </c>
+      <c r="G4" s="25" t="n">
+        <v>14917</v>
       </c>
       <c r="H4" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>0.4355517029013017</v>
+        <v>0.2279386331232653</v>
       </c>
     </row>
     <row r="5">
@@ -2053,31 +2625,31 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>General Hardware Team</t>
+          <t>Department Head - Paints</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>4067316</v>
+        <v>5391674</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>414348.7984</v>
+        <v>802339.404</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.1018727825425907</v>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>5683</v>
+        <v>0.1488108153423222</v>
+      </c>
+      <c r="G5" s="25" t="n">
+        <v>6512.5</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.165975602271912</v>
+        <v>-0.0380085199787434</v>
       </c>
     </row>
     <row r="6">
@@ -2086,31 +2658,31 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Department Head - Paints</t>
+          <t>General Hardware Team</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>3948909</v>
+        <v>5185269</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>550481.6655999999</v>
+        <v>535878.4024</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.1394009498826131</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>4888</v>
+        <v>0.103346307086479</v>
+      </c>
+      <c r="G6" s="25" t="n">
+        <v>7413.75</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>-0.2281211306541207</v>
+        <v>-0.03367415471025861</v>
       </c>
     </row>
     <row r="7">
@@ -2128,22 +2700,22 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>2614482</v>
+        <v>2964407</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>373745.8752</v>
+        <v>430440.6431999999</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0.1429521699518298</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>4791</v>
+        <v>0.1452029506069848</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>5547</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.3418320623447084</v>
+        <v>-0.5821975626151442</v>
       </c>
     </row>
     <row r="8">
@@ -2161,22 +2733,22 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1790725</v>
+        <v>2080190</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>252675.7936</v>
+        <v>317043.6716</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.1411025107707772</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>4982.25</v>
+        <v>0.1524109199640417</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>6382.25</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.1012308387786134</v>
+        <v>-0.4052007561747421</v>
       </c>
     </row>
   </sheetData>
@@ -2202,32 +2774,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>Rep Name</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="26" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="26" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="26" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="26" t="inlineStr">
         <is>
           <t>Margin %</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="26" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
@@ -2245,16 +2817,16 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>19080190</v>
+        <v>24926100</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>1096127.3724</v>
+        <v>1431524.332</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>0.05744845163491559</v>
-      </c>
-      <c r="F2" s="10" t="n">
-        <v>22251</v>
+        <v>0.0574307385431335</v>
+      </c>
+      <c r="F2" s="25" t="n">
+        <v>28702</v>
       </c>
     </row>
     <row r="3">
@@ -2269,16 +2841,16 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>155440</v>
+        <v>199210</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>24733.3112</v>
+        <v>32603.3428</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1591180597014925</v>
-      </c>
-      <c r="F3" s="10" t="n">
-        <v>114</v>
+        <v>0.1636631835751217</v>
+      </c>
+      <c r="F3" s="25" t="n">
+        <v>156</v>
       </c>
     </row>
     <row r="4">
@@ -2293,16 +2865,16 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>102600</v>
+        <v>102950</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>27921.0724</v>
+        <v>28061.734</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0.2721352085769981</v>
-      </c>
-      <c r="F4" s="10" t="n">
-        <v>234</v>
+        <v>0.272576338028169</v>
+      </c>
+      <c r="F4" s="25" t="n">
+        <v>235</v>
       </c>
     </row>
     <row r="5">
@@ -2317,16 +2889,16 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>790</v>
+        <v>1990</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>317.1556</v>
+        <v>886.9591999999999</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>0.4014627848101266</v>
-      </c>
-      <c r="F5" s="10" t="n">
-        <v>7</v>
+        <v>0.4457081407035176</v>
+      </c>
+      <c r="F5" s="25" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -2341,16 +2913,16 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>8967025</v>
+        <v>12656888</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>664793.564</v>
+        <v>952155.7472</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.07413758342371077</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>12044</v>
+        <v>0.07522826679038323</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>16912.5</v>
       </c>
     </row>
     <row r="7">
@@ -2365,16 +2937,16 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>395960</v>
+        <v>528960</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>72158.47279999999</v>
+        <v>99979.79679999998</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.1822367734114557</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>452</v>
+        <v>0.1890120175438596</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>668</v>
       </c>
     </row>
     <row r="8">
@@ -2389,16 +2961,16 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>73580</v>
+        <v>240300</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>21365.6688</v>
+        <v>63346.1152</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0.2903733188366404</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>279</v>
+        <v>0.2636126308780691</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>591</v>
       </c>
     </row>
     <row r="9">
@@ -2413,16 +2985,16 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>16460</v>
+        <v>25385</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5180.223599999999</v>
+        <v>7819.571599999999</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.314715893074119</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>152</v>
+        <v>0.3080390624384479</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>197</v>
       </c>
     </row>
     <row r="10">
@@ -2437,16 +3009,16 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>6742565</v>
+        <v>9508180</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>549397.5759999999</v>
+        <v>736651.7823999999</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>0.08148198437834858</v>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>8376</v>
+        <v>0.07747558233016202</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>12185</v>
       </c>
     </row>
     <row r="11">
@@ -2461,16 +3033,16 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1483420</v>
+        <v>1554840</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>222537.9844</v>
+        <v>238930.2808</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.1500168424316781</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>1236</v>
+        <v>0.1536687252707674</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>1391</v>
       </c>
     </row>
     <row r="12">
@@ -2485,16 +3057,16 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>180225</v>
+        <v>247935</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>58666.2228</v>
+        <v>74715.2172</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0.3255165642946317</v>
-      </c>
-      <c r="F12" s="10" t="n">
-        <v>624</v>
+        <v>0.3013500199649102</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>794</v>
       </c>
     </row>
     <row r="13">
@@ -2509,22 +3081,22 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>50050</v>
+        <v>56330</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>11493.2568</v>
+        <v>12784.4528</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.2296355004995005</v>
-      </c>
-      <c r="F13" s="10" t="n">
-        <v>400</v>
+        <v>0.2269563784839339</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>547</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -2533,22 +3105,22 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>3589596</v>
+        <v>2678479</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>331181.7516</v>
+        <v>311371.434</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>0.09226156692842313</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>5318</v>
+        <v>0.1162493467374581</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <v>4156.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -2557,22 +3129,22 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>266000</v>
+        <v>2579805</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>48733.0732</v>
+        <v>448499.3724</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>0.1832070421052631</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>265</v>
+        <v>0.1738501058800956</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>1951</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -2581,16 +3153,16 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>211720</v>
+        <v>106200</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>34433.9736</v>
+        <v>30025.1384</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0.1626392102777253</v>
-      </c>
-      <c r="F16" s="10" t="n">
-        <v>100</v>
+        <v>0.2827225838041432</v>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>299</v>
       </c>
     </row>
     <row r="17">
@@ -2601,92 +3173,92 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>GENERAL HARDWARE</t>
+          <t>ELECTRICALS</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>2295609</v>
+        <v>27190</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>246116.3416</v>
+        <v>12443.4592</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0.1072117863277239</v>
-      </c>
-      <c r="F17" s="10" t="n">
-        <v>3273</v>
+        <v>0.4576483707245311</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>PAINTS</t>
+          <t>GENERAL HARDWARE</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1535360</v>
+        <v>4696169</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>268263.688</v>
+        <v>449696.0284</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>0.1747236400583576</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>1291</v>
+        <v>0.09575805904770462</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>7037.75</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>PLUMBING</t>
+          <t>PAINTS</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>90750</v>
+        <v>274100</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>23658.1768</v>
+        <v>50412.71840000001</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.2606961630853994</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>218</v>
+        <v>0.183920898941992</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>275</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>ELECTRICALS</t>
+          <t>PLUMBING</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>27190</v>
+        <v>215000</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>12443.4592</v>
+        <v>35769.6556</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>0.4576483707245311</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>106</v>
+        <v>0.1663704911627907</v>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="21">
@@ -2701,16 +3273,16 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1796987</v>
+        <v>1898307</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>171439.7524</v>
+        <v>187738.3556</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.09540400258877776</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>2485</v>
+        <v>0.09889778397277152</v>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>2757.5</v>
       </c>
     </row>
     <row r="22">
@@ -2725,16 +3297,16 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>155000</v>
+        <v>353920</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>35623.542</v>
+        <v>59822.9632</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>0.2298293032258065</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>230</v>
+        <v>0.1690296202531646</v>
+      </c>
+      <c r="F22" s="25" t="n">
+        <v>339.5</v>
       </c>
     </row>
     <row r="23">
@@ -2749,16 +3321,16 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>619610</v>
+        <v>660200</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>158458.4128</v>
+        <v>171781.9755999999</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.2557389532125046</v>
-      </c>
-      <c r="F23" s="10" t="n">
-        <v>1902</v>
+        <v>0.260196873068767</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>2246</v>
       </c>
     </row>
     <row r="24">
@@ -2773,16 +3345,16 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>42885</v>
+        <v>51980</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>8224.168</v>
+        <v>11097.3488</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>0.1917726011425906</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>174</v>
+        <v>0.2134926664101577</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>204</v>
       </c>
     </row>
     <row r="25">
@@ -2797,16 +3369,16 @@
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>1163052</v>
+        <v>1258617</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>119199.106</v>
+        <v>136046.2384</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.1024882000116934</v>
-      </c>
-      <c r="F25" s="10" t="n">
-        <v>1762.25</v>
+        <v>0.108091848751447</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <v>1996.25</v>
       </c>
     </row>
     <row r="26">
@@ -2821,16 +3393,16 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>297736</v>
+        <v>316736</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>48961.7788</v>
+        <v>54487.9028</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>0.1644469556922911</v>
-      </c>
-      <c r="F26" s="10" t="n">
-        <v>388</v>
+        <v>0.1720293960901192</v>
+      </c>
+      <c r="F26" s="25" t="n">
+        <v>461</v>
       </c>
     </row>
     <row r="27">
@@ -2845,16 +3417,16 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>143176</v>
+        <v>204436</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>35799.2588</v>
+        <v>50118.15959999999</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.2500367296194893</v>
-      </c>
-      <c r="F27" s="10" t="n">
-        <v>472</v>
+        <v>0.245153297853607</v>
+      </c>
+      <c r="F27" s="25" t="n">
+        <v>616</v>
       </c>
     </row>
     <row r="28">
@@ -2869,16 +3441,16 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>186761</v>
+        <v>300401</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>48715.64999999999</v>
+        <v>76391.3708</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>0.2608448766070003</v>
-      </c>
-      <c r="F28" s="10" t="n">
-        <v>2360</v>
+        <v>0.2542979910186717</v>
+      </c>
+      <c r="F28" s="25" t="n">
+        <v>3309</v>
       </c>
     </row>
   </sheetData>
@@ -2904,32 +3476,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Head</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>Dept Sales</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>Dept Profit</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>Dept Margin</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="27" t="inlineStr">
         <is>
           <t>Dept Share %</t>
         </is>
@@ -2947,16 +3519,16 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>619610</v>
+        <v>660200</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>158458.4128</v>
+        <v>171781.9755999999</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>0.2557389532125046</v>
+        <v>0.260196873068767</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>0.4358352659318923</v>
+        <v>0.3715206516974194</v>
       </c>
     </row>
     <row r="3">
@@ -2971,16 +3543,16 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>1535360</v>
+        <v>2579805</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>268263.688</v>
+        <v>448499.3724</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>0.1747236400583576</v>
+        <v>0.1738501058800956</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0.3579832293288094</v>
+        <v>0.444214112922597</v>
       </c>
     </row>
     <row r="4">
@@ -2995,20 +3567,20 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>186761</v>
+        <v>300401</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>48715.64999999999</v>
+        <v>76391.3708</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0.2608448766070003</v>
+        <v>0.2542979910186717</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>0.5761809857590641</v>
+        <v>0.6484277191134441</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>GENERAL HARDWARE TEAM</t>
         </is>
@@ -3048,16 +3620,16 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>19080190</v>
+        <v>24926100</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1096127.3724</v>
+        <v>1431524.332</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.05744845163491559</v>
+        <v>0.0574307385431335</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0.4372677782874601</v>
+        <v>0.4325740150503082</v>
       </c>
     </row>
     <row r="9">
@@ -3067,16 +3639,16 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>8967025</v>
+        <v>12656888</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>664793.564</v>
+        <v>952155.7472</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.07413758342371077</v>
+        <v>0.07522826679038323</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.2055006317860625</v>
+        <v>0.2196509225350964</v>
       </c>
     </row>
     <row r="10">
@@ -3086,16 +3658,16 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>6742565</v>
+        <v>9508180</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>549397.5759999999</v>
+        <v>736651.7823999999</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.08148198437834858</v>
+        <v>0.07747558233016202</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>0.1545218584043863</v>
+        <v>0.1650074258877658</v>
       </c>
     </row>
     <row r="11">
@@ -3105,16 +3677,16 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>3589596</v>
+        <v>4696169</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>331181.7516</v>
+        <v>449696.0284</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.09226156692842313</v>
+        <v>0.09575805904770462</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.08226410050788559</v>
+        <v>0.08149853686235677</v>
       </c>
     </row>
   </sheetData>
@@ -3190,12 +3762,12 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>-16.7%</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>Outstanding! Sales 173% above team average | Margin at 5.9% below team average of 8.7% | W1→W2: Strong growth +60.1% (KES 5,631K → 9,016K) | W2→W3: Declined -48.0% (KES 9,016K → 4,692K)</t>
+          <t>+4.6%</t>
+        </is>
+      </c>
+      <c r="F2" s="29" t="inlineStr">
+        <is>
+          <t>Outstanding! Sales 169% above team average | Margin at 5.9% below team average of 8.8% | W1→W2: Strong growth +60.1% (KES 5,631K → 9,016K) | W2→W3: Declined -48.0% (KES 9,016K → 4,692K)</t>
         </is>
       </c>
     </row>
@@ -3218,12 +3790,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>+59.7%</t>
-        </is>
-      </c>
-      <c r="F3" s="14" t="inlineStr">
-        <is>
-          <t>Sales 33% above team average - solid performance | W1→W2: Strong growth +54.1% (KES 2,284K → 3,520K) | W2→W3: Steady +3.7% (KES 3,520K → 3,649K) | 📈 Consistent upward trend over 3 weeks (+59.7% overall)</t>
+          <t>+75.1%</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
+        <is>
+          <t>Sales 43% above team average - solid performance | W1→W2: Strong growth +54.1% (KES 2,284K → 3,520K) | W2→W3: Steady +3.7% (KES 3,520K → 3,649K) | W3→W4: Steady +9.6% (KES 3,649K → 3,999K)</t>
         </is>
       </c>
     </row>
@@ -3246,68 +3818,68 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>+43.6%</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>Sales 19% above team average - solid performance | W1→W2: Steady +13.1% (KES 2,371K → 2,682K) | W2→W3: Steady +26.9% (KES 2,682K → 3,403K) | 📈 Consistent upward trend over 3 weeks (+43.6% overall)</t>
+          <t>+22.8%</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>Sales 21% above team average - solid performance | W1→W2: Steady +13.1% (KES 2,371K → 2,682K) | W2→W3: Steady +26.9% (KES 2,682K → 3,403K) | W3→W4: Declined -14.5% (KES 3,403K → 2,911K)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>General Hardware Team</t>
+          <t>Department Head - Paints</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>+16.6%</t>
-        </is>
-      </c>
-      <c r="F5" s="14" t="inlineStr">
-        <is>
-          <t>Sales 43% below team average - needs improvement | W1→W2: Strong growth +35.0% (KES 1,157K → 1,561K) | W2→W3: Declined -13.6% (KES 1,561K → 1,349K) | ⚠️ Week 3 reversal after Week 2 growth - monitor closely</t>
+          <t>-3.8%</t>
+        </is>
+      </c>
+      <c r="F5" s="29" t="inlineStr">
+        <is>
+          <t>Sales 43% below team average - needs improvement | Excellent margin at 14.9% (Team avg: 8.8%) | W1→W2: Declined -13.9% (KES 1,500K → 1,292K) | W2→W3: Declined -10.4% (KES 1,292K → 1,158K)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Department Head - Paints</t>
+          <t>General Hardware Team</t>
         </is>
       </c>
       <c r="C6" s="5" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>-22.8%</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>Sales 44% below team average - needs improvement | Excellent margin at 13.9% (Team avg: 8.7%) | W1→W2: Declined -13.9% (KES 1,500K → 1,292K) | W2→W3: Declined -10.4% (KES 1,292K → 1,158K)</t>
+          <t>-3.4%</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>Sales 45% below team average - needs improvement | W1→W2: Strong growth +35.0% (KES 1,157K → 1,561K) | W2→W3: Declined -13.6% (KES 1,561K → 1,349K) | W3→W4: Declined -17.1% (KES 1,349K → 1,118K)</t>
         </is>
       </c>
     </row>
@@ -3326,16 +3898,16 @@
         <v>6</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>-34.2%</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>Sales 63% below team average - needs improvement | Excellent margin at 14.3% (Team avg: 8.7%) | W1→W2: Strong growth +46.3% (KES 838K → 1,226K) | W2→W3: Declined -55.0% (KES 1,226K → 551K)</t>
+          <t>-58.2%</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>Sales 68% below team average - needs improvement | Excellent margin at 14.5% (Team avg: 8.8%) | W1→W2: Strong growth +46.3% (KES 838K → 1,226K) | W2→W3: Declined -55.0% (KES 1,226K → 551K)</t>
         </is>
       </c>
     </row>
@@ -3354,16 +3926,16 @@
         <v>7</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>+10.1%</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>Sales 75% below team average - needs improvement | Excellent margin at 14.1% (Team avg: 8.7%) | W1→W2: Strong growth +57.8% (KES 487K → 768K) | W2→W3: Declined -30.2% (KES 768K → 536K)</t>
+          <t>-40.5%</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>Sales 78% below team average - needs improvement | Excellent margin at 15.2% (Team avg: 8.8%) | W1→W2: Strong growth +57.8% (KES 487K → 768K) | W2→W3: Declined -30.2% (KES 768K → 536K)</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3961,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>SALES REP CHARTS DATA</t>
         </is>
@@ -3429,16 +4001,16 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>19339020</v>
+        <v>25230250</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>1149098.9116</v>
+        <v>1493076.368</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0.0594186733143665</v>
+        <v>0.05917802510874843</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>22606</v>
+        <v>29108</v>
       </c>
     </row>
     <row r="5">
@@ -3448,16 +4020,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>9453025</v>
+        <v>13451533</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>763497.9292</v>
+        <v>1123301.2308</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.08076757748974535</v>
+        <v>0.08350730216399871</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>12927</v>
+        <v>18368.5</v>
       </c>
     </row>
     <row r="6">
@@ -3467,54 +4039,54 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>8456260</v>
+        <v>11367285</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>842095.0399999998</v>
+        <v>1063081.7332</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.09958244424840293</v>
+        <v>0.09352116474602334</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>10636</v>
+        <v>14917</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>4067316</v>
+        <v>5391674</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>414348.7984</v>
+        <v>802339.404</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.1018727825425907</v>
+        <v>0.1488108153423222</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>5683</v>
+        <v>6512.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>3948909</v>
+        <v>5185269</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>550481.6655999999</v>
+        <v>535878.4024</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.1394009498826131</v>
+        <v>0.103346307086479</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>4888</v>
+        <v>7413.75</v>
       </c>
     </row>
     <row r="9">
@@ -3524,16 +4096,16 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>2614482</v>
+        <v>2964407</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>373745.8752</v>
+        <v>430440.6431999999</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.1429521699518298</v>
+        <v>0.1452029506069848</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>4791</v>
+        <v>5547</v>
       </c>
     </row>
     <row r="10">
@@ -3543,16 +4115,16 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>1790725</v>
+        <v>2080190</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>252675.7936</v>
+        <v>317043.6716</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.1411025107707772</v>
+        <v>0.1524109199640417</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>4982.25</v>
+        <v>6382.25</v>
       </c>
     </row>
     <row r="15">
@@ -3563,17 +4135,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Total Sales</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Total Profit</t>
         </is>
@@ -3586,10 +4158,10 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>43635024</v>
+        <v>57622740</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3178255.464</v>
+        <v>4205183.918</v>
       </c>
     </row>
     <row r="18">
@@ -3599,10 +4171,10 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>4288916</v>
+        <v>5807571</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>721011.8503999999</v>
+        <v>984736.3771999999</v>
       </c>
     </row>
     <row r="19">
@@ -3612,10 +4184,10 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>1421661</v>
+        <v>1777021</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>360302.786</v>
+        <v>453817.9955999999</v>
       </c>
     </row>
     <row r="20">
@@ -3625,10 +4197,10 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>324136</v>
+        <v>463276</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>86373.9132</v>
+        <v>121423.1624</v>
       </c>
     </row>
     <row r="35">
@@ -3659,6 +4231,11 @@
           <t>Week 3 Sales</t>
         </is>
       </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Week 4 Sales</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -3675,6 +4252,9 @@
       <c r="D37" s="6" t="n">
         <v>4691615</v>
       </c>
+      <c r="E37" s="6" t="n">
+        <v>5891230</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -3691,6 +4271,9 @@
       <c r="D38" s="6" t="n">
         <v>3648830</v>
       </c>
+      <c r="E38" s="6" t="n">
+        <v>3998508</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -3707,37 +4290,46 @@
       <c r="D39" s="6" t="n">
         <v>3403205</v>
       </c>
+      <c r="E39" s="6" t="n">
+        <v>2911025</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B40" s="6" t="n">
-        <v>1156911</v>
+        <v>1499769</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>1561475</v>
+        <v>1291500</v>
       </c>
       <c r="D40" s="6" t="n">
-        <v>1348930</v>
+        <v>1157640</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>1442765</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B41" s="6" t="n">
-        <v>1499769</v>
+        <v>1156911</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>1291500</v>
+        <v>1561475</v>
       </c>
       <c r="D41" s="6" t="n">
-        <v>1157640</v>
+        <v>1348930</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>1117953</v>
       </c>
     </row>
     <row r="42">
@@ -3755,6 +4347,9 @@
       <c r="D42" s="6" t="n">
         <v>551240</v>
       </c>
+      <c r="E42" s="6" t="n">
+        <v>349925</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -3771,6 +4366,9 @@
       <c r="D43" s="6" t="n">
         <v>535925</v>
       </c>
+      <c r="E43" s="6" t="n">
+        <v>289465</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3780,42 +4378,42 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+      <c r="A61" s="27" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="B61" s="27" t="inlineStr">
         <is>
           <t>Gladys</t>
         </is>
       </c>
-      <c r="C61" s="12" t="inlineStr">
+      <c r="C61" s="27" t="inlineStr">
         <is>
           <t>Betha Odumo</t>
         </is>
       </c>
-      <c r="D61" s="12" t="inlineStr">
+      <c r="D61" s="27" t="inlineStr">
         <is>
           <t>Eliza</t>
         </is>
       </c>
-      <c r="E61" s="12" t="inlineStr">
+      <c r="E61" s="27" t="inlineStr">
+        <is>
+          <t>Bonface Muriu</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="inlineStr">
         <is>
           <t>Stephen</t>
         </is>
       </c>
-      <c r="F61" s="12" t="inlineStr">
-        <is>
-          <t>Bonface Muriu</t>
-        </is>
-      </c>
-      <c r="G61" s="12" t="inlineStr">
+      <c r="G61" s="27" t="inlineStr">
         <is>
           <t>Lewis</t>
         </is>
       </c>
-      <c r="H61" s="12" t="inlineStr">
+      <c r="H61" s="27" t="inlineStr">
         <is>
           <t>Bonface Kitheka</t>
         </is>
@@ -3831,22 +4429,22 @@
         <v>100</v>
       </c>
       <c r="C62" s="5" t="n">
-        <v>48.88057926409922</v>
+        <v>53.31509992964795</v>
       </c>
       <c r="D62" s="5" t="n">
-        <v>43.72641426504549</v>
+        <v>45.05419090179447</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>21.03165517177189</v>
+        <v>21.36987941062812</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>20.41938526357592</v>
+        <v>20.55179397746753</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>13.51920624726589</v>
+        <v>11.74941587974753</v>
       </c>
       <c r="H62" s="5" t="n">
-        <v>9.259647076222063</v>
+        <v>8.244825160273878</v>
       </c>
     </row>
     <row r="63">
@@ -3859,22 +4457,22 @@
         <v>100</v>
       </c>
       <c r="C63" s="5" t="n">
-        <v>66.44318617767281</v>
+        <v>75.23401045484903</v>
       </c>
       <c r="D63" s="5" t="n">
-        <v>73.28307698311806</v>
+        <v>71.20076079055589</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>36.05858418428598</v>
+        <v>53.7373319406794</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>47.90550752793872</v>
+        <v>35.89089037138923</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>32.52512655151661</v>
+        <v>28.8291109835582</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>21.98903776248255</v>
+        <v>21.23425689368355</v>
       </c>
     </row>
     <row r="64">
@@ -3887,22 +4485,22 @@
         <v>100</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>57.18393346899053</v>
+        <v>63.10464477119693</v>
       </c>
       <c r="D64" s="5" t="n">
-        <v>47.0494558966646</v>
+        <v>51.24707984059366</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>25.13934353711404</v>
+        <v>22.37357427511337</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>21.62257807661683</v>
+        <v>25.4698021162567</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>21.19348845439264</v>
+        <v>19.05661673766662</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>22.03950278687074</v>
+        <v>21.9261027896111</v>
       </c>
     </row>
     <row r="65">
@@ -3912,25 +4510,25 @@
         </is>
       </c>
       <c r="B65" s="5" t="n">
-        <v>41.56542243072535</v>
+        <v>38.82794298644105</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>56.49972121231973</v>
+        <v>54.79089174430582</v>
       </c>
       <c r="D65" s="5" t="n">
-        <v>69.66137294869951</v>
+        <v>61.36119693266583</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>71.26354400700492</v>
+        <v>97.63789587874093</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>97.51579841676183</v>
+        <v>67.80767881386812</v>
       </c>
       <c r="G65" s="5" t="n">
+        <v>95.2707001842404</v>
+      </c>
+      <c r="H65" s="5" t="n">
         <v>100</v>
-      </c>
-      <c r="H65" s="5" t="n">
-        <v>98.70609926265834</v>
       </c>
     </row>
     <row r="85">
@@ -3964,10 +4562,10 @@
         </is>
       </c>
       <c r="B87" s="5" t="n">
-        <v>19.33902</v>
+        <v>25.23025</v>
       </c>
       <c r="C87" s="5" t="n">
-        <v>1149.0989116</v>
+        <v>1493.076368</v>
       </c>
     </row>
     <row r="88">
@@ -3977,10 +4575,10 @@
         </is>
       </c>
       <c r="B88" s="5" t="n">
-        <v>9.453025</v>
+        <v>13.451533</v>
       </c>
       <c r="C88" s="5" t="n">
-        <v>763.4979292</v>
+        <v>1123.3012308</v>
       </c>
     </row>
     <row r="89">
@@ -3990,36 +4588,36 @@
         </is>
       </c>
       <c r="B89" s="5" t="n">
-        <v>8.45626</v>
+        <v>11.367285</v>
       </c>
       <c r="C89" s="5" t="n">
-        <v>842.0950399999998</v>
+        <v>1063.0817332</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Stephen</t>
+          <t>Bonface Muriu</t>
         </is>
       </c>
       <c r="B90" s="5" t="n">
-        <v>4.067316</v>
+        <v>5.391674</v>
       </c>
       <c r="C90" s="5" t="n">
-        <v>414.3487984</v>
+        <v>802.3394039999999</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>Bonface Muriu</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B91" s="5" t="n">
-        <v>3.948909</v>
+        <v>5.185269</v>
       </c>
       <c r="C91" s="5" t="n">
-        <v>550.4816655999999</v>
+        <v>535.8784024</v>
       </c>
     </row>
     <row r="92">
@@ -4029,10 +4627,10 @@
         </is>
       </c>
       <c r="B92" s="5" t="n">
-        <v>2.614482</v>
+        <v>2.964407</v>
       </c>
       <c r="C92" s="5" t="n">
-        <v>373.7458751999999</v>
+        <v>430.4406432</v>
       </c>
     </row>
     <row r="93">
@@ -4042,10 +4640,10 @@
         </is>
       </c>
       <c r="B93" s="5" t="n">
-        <v>1.790725</v>
+        <v>2.08019</v>
       </c>
       <c r="C93" s="5" t="n">
-        <v>252.6757936</v>
+        <v>317.0436716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>